<commit_message>
data: extrair contratação PNCP específica
</commit_message>
<xml_diff>
--- a/EDITAIS/CONTRATACAO-00394502000144-2026-14259/contratacao-completa.xlsx
+++ b/EDITAIS/CONTRATACAO-00394502000144-2026-14259/contratacao-completa.xlsx
@@ -668,7 +668,7 @@
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2026-10-22T21:24:06+00:00</t>
+          <t>2026-10-22T22:20:34+00:00</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,11 @@
           <t>3.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>239,00</t>
@@ -808,7 +812,11 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>138,08</t>
@@ -848,7 +856,11 @@
           <t>3.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>265,50</t>
@@ -888,7 +900,11 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>503,70</t>
@@ -928,7 +944,11 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>198,00</t>
@@ -968,7 +988,11 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>485,27</t>
@@ -1008,7 +1032,11 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>2370,45</t>
@@ -1048,7 +1076,11 @@
           <t>5.0</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>394,20</t>
@@ -1088,7 +1120,11 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>892,06</t>
@@ -1128,7 +1164,11 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>4232,54</t>
@@ -1168,7 +1208,11 @@
           <t>4.0</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>36,92</t>
@@ -1208,7 +1252,11 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>206,90</t>
@@ -1248,7 +1296,11 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>1518,14</t>
@@ -1288,7 +1340,11 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>3071,84</t>
@@ -1326,10 +1382,10 @@
   <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1355,184 +1411,664 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:44:36</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:44:36</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dispensa Eletronica N165. Mat. GVA S-3_Assinatura_01.pdf</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:37</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:37</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:37</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:38</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:39</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:38</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:38</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:38</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:37</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ANEXO_I_-_FORMALIZACAO_DE_DEMANDA_assinado-1.pdf</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:40</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Retificação</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Alteração do item devido a mudança de situação para Em Andamento</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-22T17:45:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Inclusão</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Item de Contratação</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Compras.gov.br</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D31"/>
@@ -1546,10 +2082,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1573,7 +2109,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>COMPLETO</t>
+          <t>PARCIAL</t>
         </is>
       </c>
     </row>
@@ -1585,7 +2121,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22T21:24:06+00:00</t>
+          <t>2026-10-22T22:20:34+00:00</t>
         </is>
       </c>
     </row>
@@ -1645,79 +2181,139 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>["https://pncp.gov.br/api/pncp/v1/orgaos/00394502000144/compras/2026/14259", "https://pncp.gov.br/api/pncp/v1/orgaos/00394502000144/compras/2026/14259/itens", "https://pncp.gov.br/api/pncp/v1/orgaos/00394502000144/compras/2026/14259/historico"]</t>
+          <t>{"geral": "https://pncp.gov.br/api/consulta/v1/orgaos/00394502000144/compras/2026/14259", "itens": "https://pncp.gov.br/api/pncp/v1/orgaos/00394502000144/compras/2026/14259/itens", "eventos": "https://pncp.gov.br/api/pncp/v1/orgaos/00394502000144/compras/2026/14259/historico", "fallback_geral": "https://pncp.gov.br/api/consulta/v1/contratacoes/proposta"}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>base_api</t>
+          <t>fonte_dados_gerais</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/api/pncp</t>
+          <t>consulta_detalhe</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>documentacao_api</t>
+          <t>base_api_consulta</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/manual/pt-br/latest/contratacao/consultar_historico_da_contratacao.html</t>
+          <t>https://pncp.gov.br/api/consulta/v1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>erros_por_endpoint</t>
+          <t>base_api_itens_historico</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>https://pncp.gov.br/api/pncp/v1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>quantidade_itens</t>
+          <t>documentacao_api_consulta</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>https://pncp.gov.br/api/consulta/swagger-ui/index.html</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>quantidade_eventos</t>
+          <t>documentacao_api_itens_historico</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>https://pncp.gov.br/manual/pt-br/latest/contratacao/consultar_historico_da_contratacao.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>erros_por_endpoint</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>{"geral": "Detalhe: HTTP 404 em https://pncp.gov.br/api/consulta/v1/orgaos/00394502000144/compras/2026/14259; fallback de propostas: Contratação 00394502000144-1-014259/2026 não localizada nas rotas públicas alternativas. proposta_cnpj_janela: páginas=5; registros=244; amostras=['00394502000144-1-003337/2026', '00394502000144-1-013399/2026', '00394502000144-1-013455/2026', '00394502000144-1-013637/2026'] | proposta_cnpj_sem_modalidade_janela: páginas=5; registros=250; amostras=['00394502000144-1-000002/2026', '00394502000144-1-000251/2025', '00394502000144-1-001378/2025', '00394502000144-1-000020/2026'] | proposta_cnpj: falha na página 2: HTTP 429 em https://pncp.gov.br/api/consulta/v1/contratacoes/proposta?dataFinal=20271022&amp;cnpj=00394502000144&amp;tamanhoPagina=50&amp;pagina=2 | proposta_cnpj: páginas=1; registros=50; amostras=['00394502000144-1-000002/2026', '00394502000144-1-000251/2025', '00394502000144-1-001378/2025', '00394502000144-1-000020/2026']"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>avisos_por_endpoint</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>{"geral_detalhe": "HTTP 404 em https://pncp.gov.br/api/consulta/v1/orgaos/00394502000144/compras/2026/14259"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>quantidade_itens</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>quantidade_eventos</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>quantidade_itens_esperada</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Os campos são preenchidos com os valores efetivamente devolvidos pela API; campos ausentes permanecem vazios. A extração deve ser comparada à página pública se o PNCP alterar o esquema dos endpoints.</t>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Os campos usam somente dados retornados pela API oficial. A consulta geral usa a rota de detalhe e, se ela retornar 404, procura o identificador PNCP exato nas listas oficiais. A consulta alternativa pesquisa uma janela de publicação com e sem filtro de modalidade, para reduzir paginação e respeitar os códigos publicados pelo PNCP. A extração só é marcada COMPLETO quando dados gerais válidos, 14 itens com unidade e histórico com dados são recuperados.</t>
         </is>
       </c>
     </row>

</xml_diff>